<commit_message>
Add 12 pre-seed/angel investors to Workstream 2; add HTML dashboard view
Expands Workstream 2 from 14 to 26 qualified investors (50 opportunities total),
each vetted for explicit pre-seed / pre-revenue appetite and health/AI fit:
Nina Capital, 2048 Ventures, January Ventures, Afore Capital, Air Street Capital,
Village Global, Y Combinator (Eligible); Zetta, AIX, Susa, Broadway Angels
(Researching); Basis Set (low-priority). Each row carries check size, route
(cold vs warm intro), fit score, hours, next action, and a verification comment.

Adds funding_dashboard.html — a read-only, theme-aware view generated from the
workbook (summary tiles, application calendar, and the full pipeline grouped by
workstream). The xlsx remains the single source of truth; regenerate the page
from it rather than editing the HTML by hand.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Uh1jFHPZFJnmJ5vxj2WzQC
</commit_message>
<xml_diff>
--- a/Funding_Dashboard.xlsx
+++ b/Funding_Dashboard.xlsx
@@ -500,6 +500,78 @@
 Search-verified via official-domain content (coefficientgiving.org) on 2026-08-11 (WebSearch). Direct official-page fetch was BLOCKED by this session's egress policy, so this is NOT a live-page confirmation. Confirm on the official page before relying. Source: https://coefficientgiving.org/funds/global-health-wellbeing-opportunities/request-for-proposals-global-health-and-wellbeing-in-an-era-of-transformative-ai/</t>
       </text>
     </comment>
+    <comment ref="J40" authorId="0" shapeId="0">
+      <text>
+        <t>First check ~$1-3M (seed); pre-seed done selectively.
+Search-verified via official-domain content (www.zettavp.com) on 2026-08-11 (WebSearch). Direct official-page fetch was BLOCKED by this session's egress policy - NOT a live-page confirmation. Confirm before relying. Source: https://www.zettavp.com/</t>
+      </text>
+    </comment>
+    <comment ref="J41" authorId="0" shapeId="0">
+      <text>
+        <t>EUR250K-EUR1.5M initial (EUR-denominated fund).
+Search-verified via official-domain content (www.nina.capital) on 2026-08-11 (WebSearch). Direct official-page fetch was BLOCKED by this session's egress policy - NOT a live-page confirmation. Confirm before relying. Source: https://www.nina.capital/</t>
+      </text>
+    </comment>
+    <comment ref="J42" authorId="0" shapeId="0">
+      <text>
+        <t>$250K-$750K (Fast Track); up to $3M broader pre-seed/seed.
+Search-verified via official-domain content (www.2048.vc) on 2026-08-11 (WebSearch). Direct official-page fetch was BLOCKED by this session's egress policy - NOT a live-page confirmation. Confirm before relying. Source: https://www.2048.vc/</t>
+      </text>
+    </comment>
+    <comment ref="J43" authorId="0" shapeId="0">
+      <text>
+        <t>$750K-$3M initial.
+Search-verified via official-domain content (www.aixventures.com) on 2026-08-11 (WebSearch). Direct official-page fetch was BLOCKED by this session's egress policy - NOT a live-page confirmation. Confirm before relying. Source: https://www.aixventures.com/</t>
+      </text>
+    </comment>
+    <comment ref="J44" authorId="0" shapeId="0">
+      <text>
+        <t>$250K-$500K (pre-seed, selective).
+Search-verified via official-domain content (www.basisset.com) on 2026-08-11 (WebSearch). Direct official-page fetch was BLOCKED by this session's egress policy - NOT a live-page confirmation. Confirm before relying. Source: https://www.basisset.com/</t>
+      </text>
+    </comment>
+    <comment ref="J45" authorId="0" shapeId="0">
+      <text>
+        <t>$500K-$5M at pre-seed/seed.
+Search-verified via official-domain content (www.airstreet.com) on 2026-08-11 (WebSearch). Direct official-page fetch was BLOCKED by this session's egress policy - NOT a live-page confirmation. Confirm before relying. Source: https://www.airstreet.com/</t>
+      </text>
+    </comment>
+    <comment ref="J46" authorId="0" shapeId="0">
+      <text>
+        <t>$500,000 standard SAFE ($125K/7% + $375K uncapped).
+Search-verified via official-domain content (www.ycombinator.com) on 2026-08-11 (WebSearch). Direct official-page fetch was BLOCKED by this session's egress policy - NOT a live-page confirmation. Confirm before relying. Source: https://www.ycombinator.com/apply</t>
+      </text>
+    </comment>
+    <comment ref="J47" authorId="0" shapeId="0">
+      <text>
+        <t>$50K-$2M+ (flexible pre-seed range).
+Search-verified via official-domain content (www.afore.vc) on 2026-08-11 (WebSearch). Direct official-page fetch was BLOCKED by this session's egress policy - NOT a live-page confirmation. Confirm before relying. Source: https://www.afore.vc/pitch</t>
+      </text>
+    </comment>
+    <comment ref="J48" authorId="0" shapeId="0">
+      <text>
+        <t>$500K-$2M (pre-seed); $1-3M seed.
+Search-verified via official-domain content (www.susaventures.com) on 2026-08-11 (WebSearch). Direct official-page fetch was BLOCKED by this session's egress policy - NOT a live-page confirmation. Confirm before relying. Source: https://www.susaventures.com/</t>
+      </text>
+    </comment>
+    <comment ref="J49" authorId="0" shapeId="0">
+      <text>
+        <t>$500K-$3M (Velocity pre-seed up to $1M).
+Search-verified via official-domain content (www.villageglobal.com) on 2026-08-11 (WebSearch). Direct official-page fetch was BLOCKED by this session's egress policy - NOT a live-page confirmation. Confirm before relying. Source: https://www.villageglobal.com/velocity</t>
+      </text>
+    </comment>
+    <comment ref="J50" authorId="0" shapeId="0">
+      <text>
+        <t>$150K-$500K.
+Search-verified via official-domain content (www.january.ventures) on 2026-08-11 (WebSearch). Direct official-page fetch was BLOCKED by this session's egress policy - NOT a live-page confirmation. Confirm before relying. Source: https://www.january.ventures/</t>
+      </text>
+    </comment>
+    <comment ref="J51" authorId="0" shapeId="0">
+      <text>
+        <t>~$5K-$50K per group; members join larger rounds.
+Search-verified via official-domain content (www.broadway-angels.com) on 2026-08-11 (WebSearch). Direct official-page fetch was BLOCKED by this session's egress policy - NOT a live-page confirmation. Confirm before relying. Source: https://www.broadway-angels.com/</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -905,7 +977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O39"/>
+  <dimension ref="A1:O51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3647,6 +3719,849 @@
       <c r="O39" s="5" t="inlineStr">
         <is>
           <t>https://coefficientgiving.org/funds/global-health-wellbeing-opportunities/request-for-proposals-global-health-and-wellbeing-in-an-era-of-transformative-ai/</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>2</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Zetta Venture Partners</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Zetta Venture Partners</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>US / Europe - SF</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>AI-native B2B only (AI/ML must be the core product, not a feature); pre-seed named but sweet spot is seed. HealthTech in scope. Must be framed as core-ML (drift/performance monitoring), not a compliance wrapper. Cold route unconfirmed - likely warm intro.</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>4</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>3-6</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Researching</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Confirm the submission channel on zettavp.com and frame the product as core-ML; warm intro via CHAI / health-AI operators.</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>https://www.zettavp.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Nina Capital</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Nina Capital</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Europe / North America - Barcelona</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Healthcare-only fund with explicit pre-seed appetite; invests in North America. 'Need-driven' healthtech + AI/ML thesis = strongest thematic match. No drugs/vaccines. Open cold route.</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>5</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Submit the pitch deck to dealflow@nina.capital (healthcare-only pre-seed; strongest thematic fit of the new batch).</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>https://www.nina.capital/</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>2</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2048 Ventures</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2048 Ventures</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>US - Boston / NYC</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>750000</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Pre-seed / first-round fund based in Boston + NYC. Health + Vertical-AI thesis. Pre-Seed Fast Track is cold (no warm intro), decision in ~10 business days. Eligible if not already raised &gt;$2M (SafeAI qualifies). Pre-incorporation acceptable.</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>5</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Apply via the Pre-Seed Fast Track form at 2048.vc (Boston-based; cold route; ~10-business-day decision).</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>https://www.2048.vc/</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>2</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>AIX Ventures</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>AIX Ventures</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>US - SF</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>AI-native only (AI must be the core competitive advantage); healthcare interest stated. Practitioner GPs scrutinise the technical AI core - must show proprietary ML (drift/performance monitoring), not process tooling. Warm intro strongly favoured.</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>4</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Researching</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Secure an academic-AI / CHAI warm intro; lead with proprietary-ML defensibility (not compliance tooling).</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>https://www.aixventures.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>2</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Basis Set Ventures</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Basis Set Ventures</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>US - SF</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>AI/ML for productivity &amp; infrastructure; healthcare is NOT a stated thesis. Pre-seed done selectively/secondarily. Marginal fit - only if framed as enterprise-AI automation for health systems. Low priority.</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>2</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Researching</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Low priority; only pursue if framing SafeAI as enterprise-AI automation. Cold note via basisset.com.</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>https://www.basisset.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>2</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Air Street Capital</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Air Street Capital</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>US / Europe - London</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>AI-first fund incl. TechBio / AI-native life sciences; made a 2025 healthcare deal. Explicit pre-seed/seed ($500K-$5M). Solo-GP, thesis-driven - AI-capability narrative matters more than traction. Direct cold-email route.</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>4</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Email Nathan Benaich (nathan@airstreet.com) with the core AI capability + stage; a CHAI / academic-AI intro warms it.</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>https://www.airstreet.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>2</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Y Combinator</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Y Combinator</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Global - SF batch</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>500000</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Pre-seed accelerator; accepts pre-revenue/idea-stage and pre-incorporation founders. Standard DILUTIVE deal: $125K for 7% + $375K uncapped SAFE (~$500K, ~9-10% total). Deep clinical-AI portfolio. In-person SF batch = relocation. Founder must hold &gt;=10% equity. Batch deadlines.</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>4</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Batch-based (next window; Fall 2026 closed 27 Jul 2026)</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>8-15</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Target the next batch (Fall 2026 deadline passed); complete the cold application at ycombinator.com/apply. Weigh SF relocation + ~10% dilution.</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>https://www.ycombinator.com/apply</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>2</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Afore Capital</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Afore Capital</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>US - SF</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Dedicated pre-seed / pre-formation fund (backs founders before traction; pre-incorporation acceptable). Health + AI in scope; founder-conviction weighted over market analysis. Open cold pitch form; fast decisions.</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>5</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Submit the cold pitch form at afore.vc/pitch; lead with the Harvard DrPH founder story.</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>https://www.afore.vc/pitch</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>2</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Susa Ventures</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Susa Ventures</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>US - SF</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Pre-seed stated but seed-weighted (leads seed rounds). AI + healthcare + digital health named sectors. May expect more formation/traction than a pure pre-seed fund. Warm intro preferred; cold mechanism unconfirmed.</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>3</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Researching</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Confirm they'll write a first pre-incorporation check; route a warm intro via CHAI / HealthLab or a digital-health portfolio founder.</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>https://www.susaventures.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>2</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Village Global</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Village Global</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Network-driven pre-seed/seed ($500K-$3M); the Velocity pre-seed program invests up to $1M with 'particular depth in healthcare.' Referral-preferred but a form + hello@villageglobal.vc exist. Pre-incorporation OK.</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>4</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Seek an intro via a Village Global Network Leader / portfolio founder; otherwise apply through the Velocity form.</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>https://www.villageglobal.com/velocity</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>2</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>January Ventures</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>January Ventures</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>US / Europe - Boston</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>500000</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Pre-seed fund that explicitly invests BEFORE product/customers/revenue - ideal for a pre-incorporation company. Boston + London. B2B incl. digital health; female / underdog-founder thesis. Cold ~2-minute form, no deck or warm intro needed (lowest-friction route of the batch).</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>5</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Eligible</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Complete the ~2-minute cold form at january.ventures (Boston; no deck required; pre-product mandate fits SafeAI).</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>https://www.january.ventures/</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>2</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Broadway Angels</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Broadway Angels</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Investor</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>US - SF</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>50000</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>All-female group of VC GPs &amp; senior tech execs; pre-seed/seed, digital health + IT, receptive to women founders. Small checks (~$5K-$50K) but high-signal network / follow-on value. No public form - warm intro required.</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>3</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Rolling</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>3-6</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Researching</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>Lara</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Map the shortest warm-intro path (Signal/nfx) via CHAI / i-Lab mentors; no cold route exists.</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>https://www.broadway-angels.com/</t>
         </is>
       </c>
     </row>

</xml_diff>